<commit_message>
Deploy Atlas site from 39f0ba0e1cdd0af37ae15de40d22a02d3824d4c0
</commit_message>
<xml_diff>
--- a/downloads/formulas/project-quantitative-methods.xlsx
+++ b/downloads/formulas/project-quantitative-methods.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Formula Reference" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1669,7 +1669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2480,9 +2480,41 @@
         </is>
       </c>
     </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>FRM-COM-001</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Potential communication channels</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>C = n(n - 1) / 2</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Potential pairwise paths.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>supplemental_official_pmi</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>n is an integer of at least 1; direction is not counted separately; the measure represents potential interpersonal paths rather than messages, technologies, methods, or required direct communications.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <autoFilter ref="A1:F27"/>
+  <autoFilter ref="A1:F28"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Deploy Atlas site from dbf72007c039e5fc5ed405aaecd6d04782031fd9
</commit_message>
<xml_diff>
--- a/downloads/formulas/project-quantitative-methods.xlsx
+++ b/downloads/formulas/project-quantitative-methods.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Formula Reference" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1669,7 +1669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2291,17 +2291,17 @@
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-007</t>
+          <t>FRM-EVM-010</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>EAC — remaining work at original rate</t>
+          <t>Variance at completion</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>EAC = AC + (BAC - EV)</t>
+          <t>VAC = BAC - EAC</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2316,93 +2316,93 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Past variance is atypical and remaining work will perform at the original budgeted rate.</t>
+          <t>BAC and EAC cover the same measured scope.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-008</t>
+          <t>FRM-EVM-011</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>EAC — cost and schedule influence remaining work</t>
+          <t>To-complete performance index against BAC</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>EAC = AC + ((BAC - EV) / (CPI × SPI))</t>
+          <t>TCPI(BAC) = (BAC - EV) / (BAC - AC)</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Currency.</t>
+          <t>Dimensionless ratio.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>verified_current_course</t>
+          <t>supplemental_official_pmi</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Both current cost and schedule performance are expected to influence remaining cost; CPI and SPI are nonzero.</t>
+          <t>BAC minus AC is positive and BAC remains the selected target.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-009</t>
+          <t>FRM-EVM-012</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>EAC — bottom-up remaining estimate</t>
+          <t>To-complete performance index against approved EAC</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>EAC = AC + bottom-up ETC</t>
+          <t>TCPI(EAC) = (BAC - EV) / (EAC - AC)</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Currency.</t>
+          <t>Dimensionless ratio.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>verified_current_course</t>
+          <t>supplemental_official_pmi</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>The original estimate is no longer reliable and the remaining work has been re-estimated.</t>
+          <t>EAC minus AC is positive and EAC is the selected approved target.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-010</t>
+          <t>FRM-COM-001</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Variance at completion</t>
+          <t>Potential communication channels</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>VAC = BAC - EAC</t>
+          <t>C = n(n - 1) / 2</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Currency.</t>
+          <t>Potential pairwise paths.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -2411,102 +2411,6 @@
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>BAC and EAC cover the same measured scope.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="34" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>FRM-EVM-011</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>To-complete performance index against BAC</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>TCPI(BAC) = (BAC - EV) / (BAC - AC)</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Dimensionless ratio.</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>supplemental_official_pmi</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>BAC minus AC is positive and BAC remains the selected target.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="34" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>FRM-EVM-012</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>To-complete performance index against approved EAC</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>TCPI(EAC) = (BAC - EV) / (EAC - AC)</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>Dimensionless ratio.</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>supplemental_official_pmi</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>EAC minus AC is positive and EAC is the selected approved target.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>FRM-COM-001</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Potential communication channels</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>C = n(n - 1) / 2</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Potential pairwise paths.</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>supplemental_official_pmi</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>n is an integer of at least 1; direction is not counted separately; the measure represents potential interpersonal paths rather than messages, technologies, methods, or required direct communications.</t>
         </is>
@@ -2514,7 +2418,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <autoFilter ref="A1:F28"/>
+  <autoFilter ref="A1:F25"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
Deploy Atlas site from 2806ff20d8671fa7de1a23e3e9722566fe344397
</commit_message>
<xml_diff>
--- a/downloads/formulas/project-quantitative-methods.xlsx
+++ b/downloads/formulas/project-quantitative-methods.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Formula Reference" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Formula Reference'!$A$1:$F$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1232,7 +1232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1258,7 +1258,7 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>ServiceBridge Modernization status-date example.</t>
+          <t>ServiceBridge Modernization: choose EAC from the forecast assumption, not a memorized preference.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1299,7 +1299,7 @@
       <c r="C5" s="2" t="n"/>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Interpretation</t>
+          <t>Formula-selection guidance</t>
         </is>
       </c>
       <c r="E5" s="2" t="n"/>
@@ -1317,7 +1317,7 @@
       <c r="C6" s="2" t="n"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>EV is below PV and AC exceeds EV. If current CPI continues, forecast total cost is above BAC. SV is in dollars, not days.</t>
+          <t>CPI continues: demonstrated cost efficiency persists. Original planned rate: current variance will not continue. Bottom-up ETC: original estimate is no longer reliable and remaining work is re-estimated. CPI × SPI: both cost and schedule performance influence remaining work. SPI is dimensionless, not a monetary measure. The last three cases are S3 supplemental PMI support, not July 2026 course-verified formulas.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -1352,19 +1352,21 @@
       <c r="F8" s="2" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Bottom-up ETC</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>1600000</v>
+      </c>
       <c r="C9" s="2" t="n"/>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Calculated measures</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="n"/>
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
@@ -1372,15 +1374,12 @@
       <c r="F10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="B11" s="11">
-        <f>B7-B6</f>
-        <v/>
-      </c>
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Calculated measures and EAC alternatives</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n"/>
       <c r="C11" s="2" t="n"/>
       <c r="D11" s="2" t="n"/>
       <c r="E11" s="2" t="n"/>
@@ -1389,11 +1388,11 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>SPI</t>
-        </is>
-      </c>
-      <c r="B12" s="12">
-        <f>IFERROR(B7/B6,"")</f>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
+        <f>B7-B6</f>
         <v/>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -1404,11 +1403,11 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>CV</t>
-        </is>
-      </c>
-      <c r="B13" s="11">
-        <f>B7-B8</f>
+          <t>SPI</t>
+        </is>
+      </c>
+      <c r="B13" s="12">
+        <f>IFERROR(B7/B6,"")</f>
         <v/>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -1419,11 +1418,11 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>CPI</t>
-        </is>
-      </c>
-      <c r="B14" s="12">
-        <f>IFERROR(B7/B8,"")</f>
+          <t>CV</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>B7-B8</f>
         <v/>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -1434,11 +1433,11 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>EAC (CPI continues)</t>
-        </is>
-      </c>
-      <c r="B15" s="11">
-        <f>IFERROR(B5/B14,"")</f>
+          <t>CPI</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>IFERROR(B7/B8,"")</f>
         <v/>
       </c>
       <c r="C15" s="2" t="n"/>
@@ -1446,29 +1445,33 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="n"/>
     </row>
-    <row r="16">
+    <row r="16" ht="34" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ETC</t>
+          <t>EAC · CPI continues</t>
         </is>
       </c>
       <c r="B16" s="11">
-        <f>B15-B8</f>
+        <f>IFERROR(B5/B15,"")</f>
         <v/>
       </c>
       <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Source status: Process Groups: A Practice Guide, Table 10-1, printed page 311. The July 2026 course independently supports only EAC = BAC / CPI. Yellow cells are editable; Bottom-up ETC is an explicit separate input.</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="34" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>VAC</t>
+          <t>EAC · original planned rate</t>
         </is>
       </c>
       <c r="B17" s="11">
-        <f>B5-B15</f>
+        <f>B8+(B5-B7)</f>
         <v/>
       </c>
       <c r="C17" s="2" t="n"/>
@@ -1476,14 +1479,14 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="n"/>
     </row>
-    <row r="18">
+    <row r="18" ht="34" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TCPI (BAC)</t>
-        </is>
-      </c>
-      <c r="B18" s="12">
-        <f>IFERROR((B5-B7)/(B5-B8),"")</f>
+          <t>EAC · new bottom-up ETC</t>
+        </is>
+      </c>
+      <c r="B18" s="11">
+        <f>B8+B9</f>
         <v/>
       </c>
       <c r="C18" s="2" t="n"/>
@@ -1491,14 +1494,14 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="34" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TCPI (EAC)</t>
-        </is>
-      </c>
-      <c r="B19" s="12">
-        <f>IFERROR((B5-B7)/(B15-B8),"")</f>
+          <t>EAC · CPI × SPI influence</t>
+        </is>
+      </c>
+      <c r="B19" s="11">
+        <f>IFERROR(B8+(B5-B7)/(B15*B13),"")</f>
         <v/>
       </c>
       <c r="C19" s="2" t="n"/>
@@ -1506,14 +1509,75 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ETC · CPI case</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
+        <f>B16-B8</f>
+        <v/>
+      </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VAC · CPI case</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>B5-B16</f>
+        <v/>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TCPI (BAC)</t>
+        </is>
+      </c>
+      <c r="B22" s="12">
+        <f>IFERROR((B5-B7)/(B5-B8),"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TCPI (EAC · CPI case)</t>
+        </is>
+      </c>
+      <c r="B23" s="12">
+        <f>IFERROR((B5-B7)/(B16-B8),"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="D6:F14"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="D6:F10"/>
+    <mergeCell ref="D16:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1669,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2291,17 +2355,17 @@
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-010</t>
+          <t>FRM-EVM-007</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Variance at completion</t>
+          <t>EAC — remaining work at original rate</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>VAC = BAC - EAC</t>
+          <t>EAC = AC + (BAC - EV)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2316,29 +2380,29 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>BAC and EAC cover the same measured scope.</t>
+          <t>Current variance is not expected to continue; remaining work is expected to be accomplished at the originally planned rate.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="34" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-011</t>
+          <t>FRM-EVM-008</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>To-complete performance index against BAC</t>
+          <t>EAC — cost and schedule influence remaining work</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>TCPI(BAC) = (BAC - EV) / (BAC - AC)</t>
+          <t>EAC = AC + ((BAC - EV) / (CPI × SPI))</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Dimensionless ratio.</t>
+          <t>Currency.</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -2348,29 +2412,29 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>BAC minus AC is positive and BAC remains the selected target.</t>
+          <t>Both current cost and schedule performance are expected to influence remaining cost; CPI and SPI are nonzero.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="34" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>FRM-EVM-012</t>
+          <t>FRM-EVM-009</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>To-complete performance index against approved EAC</t>
+          <t>EAC — bottom-up remaining estimate</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>TCPI(EAC) = (BAC - EV) / (EAC - AC)</t>
+          <t>EAC = AC + bottom-up ETC</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Dimensionless ratio.</t>
+          <t>Currency.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -2380,37 +2444,133 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>EAC minus AC is positive and EAC is the selected approved target.</t>
+          <t>The original estimate is no longer valid or reliable; the remaining work receives a new detailed bottom-up estimate.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="34" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>FRM-EVM-010</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Variance at completion</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>VAC = BAC - EAC</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Currency.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>supplemental_official_pmi</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>BAC and EAC cover the same measured scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>FRM-EVM-011</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>To-complete performance index against BAC</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>TCPI(BAC) = (BAC - EV) / (BAC - AC)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Dimensionless ratio.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>supplemental_official_pmi</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>BAC minus AC is positive and BAC remains the selected target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>FRM-EVM-012</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>To-complete performance index against approved EAC</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>TCPI(EAC) = (BAC - EV) / (EAC - AC)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Dimensionless ratio.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>supplemental_official_pmi</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>EAC minus AC is positive and EAC is the selected approved target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>FRM-COM-001</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Potential communication channels</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>C = n(n - 1) / 2</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Potential pairwise paths.</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>supplemental_official_pmi</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>n is an integer of at least 1; direction is not counted separately; the measure represents potential interpersonal paths rather than messages, technologies, methods, or required direct communications.</t>
         </is>
@@ -2418,7 +2578,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <autoFilter ref="A1:F25"/>
+  <autoFilter ref="A1:F28"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>